<commit_message>
Translate report, model and data to English
</commit_message>
<xml_diff>
--- a/Data/sales_targets_monthly.xlsx
+++ b/Data/sales_targets_monthly.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI按月" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原始数据" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI by Month" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Data" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -423,7 +423,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>月份日期</t>
+          <t>Month Date</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -433,27 +433,27 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>年份</t>
+          <t>Year</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>月份</t>
+          <t>Month</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>销售人员</t>
+          <t>Salesperson</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>KPI目标</t>
+          <t>KPI Target</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>公司</t>
+          <t>Company</t>
         </is>
       </c>
     </row>
@@ -474,11 +474,11 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Lei He (Lina)</t>
+          <t>Cathy Kong</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>40000</v>
+        <v>25000</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -503,11 +503,11 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Lei He (Lina)</t>
+          <t>Cathy Kong</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>35000</v>
+        <v>20000</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -532,11 +532,11 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Lei He (Lina)</t>
+          <t>Cathy Kong</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>35000</v>
+        <v>25000</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -561,11 +561,11 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Lei He (Lina)</t>
+          <t>Cathy Kong</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>40000</v>
+        <v>30000</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -590,11 +590,11 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Lei He (Lina)</t>
+          <t>Cathy Kong</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>40000</v>
+        <v>25000</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -619,11 +619,11 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Lei He (Lina)</t>
+          <t>Cathy Kong</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>40000</v>
+        <v>25000</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -648,11 +648,11 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Lei He (Lina)</t>
+          <t>Cathy Kong</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>35000</v>
+        <v>25000</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -677,11 +677,11 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Lei He (Lina)</t>
+          <t>Cathy Kong</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>35000</v>
+        <v>25000</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -706,11 +706,11 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Lei He (Lina)</t>
+          <t>Cathy Kong</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>40000</v>
+        <v>25000</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -735,11 +735,11 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Lei He (Lina)</t>
+          <t>Cathy Kong</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>40000</v>
+        <v>20000</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -764,11 +764,11 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Lei He (Lina)</t>
+          <t>Cathy Kong</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>40000</v>
+        <v>25000</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -793,11 +793,11 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Lei He (Lina)</t>
+          <t>Cathy Kong</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>40000</v>
+        <v>25000</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -822,11 +822,11 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Ting Qin (Joyce)</t>
+          <t>YUN CHU</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>100000</v>
+        <v>80000</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -851,11 +851,11 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Ting Qin (Joyce)</t>
+          <t>YUN CHU</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>100000</v>
+        <v>80000</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -880,11 +880,11 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Ting Qin (Joyce)</t>
+          <t>YUN CHU</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>105000</v>
+        <v>75000</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -909,11 +909,11 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Ting Qin (Joyce)</t>
+          <t>YUN CHU</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>95000</v>
+        <v>80000</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -938,11 +938,11 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Ting Qin (Joyce)</t>
+          <t>YUN CHU</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>95000</v>
+        <v>80000</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -967,11 +967,11 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Ting Qin (Joyce)</t>
+          <t>YUN CHU</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>90000</v>
+        <v>70000</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -996,11 +996,11 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Ting Qin (Joyce)</t>
+          <t>YUN CHU</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>100000</v>
+        <v>75000</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1025,11 +1025,11 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Ting Qin (Joyce)</t>
+          <t>YUN CHU</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>90000</v>
+        <v>80000</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1054,11 +1054,11 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Ting Qin (Joyce)</t>
+          <t>YUN CHU</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>105000</v>
+        <v>85000</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1083,11 +1083,11 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Ting Qin (Joyce)</t>
+          <t>YUN CHU</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>90000</v>
+        <v>75000</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1112,11 +1112,11 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Ting Qin (Joyce)</t>
+          <t>YUN CHU</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>105000</v>
+        <v>75000</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1141,11 +1141,11 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Ting Qin (Joyce)</t>
+          <t>YUN CHU</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>100000</v>
+        <v>70000</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1170,11 +1170,11 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Qiang Han (Irene)</t>
+          <t>JIE ZOU</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1199,11 +1199,11 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Qiang Han (Irene)</t>
+          <t>JIE ZOU</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1228,11 +1228,11 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Qiang Han (Irene)</t>
+          <t>JIE ZOU</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>45000</v>
+        <v>55000</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1257,11 +1257,11 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Qiang Han (Irene)</t>
+          <t>JIE ZOU</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>45000</v>
+        <v>50000</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1286,11 +1286,11 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Qiang Han (Irene)</t>
+          <t>JIE ZOU</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>55000</v>
+        <v>60000</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1315,11 +1315,11 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Qiang Han (Irene)</t>
+          <t>JIE ZOU</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>45000</v>
+        <v>65000</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1344,11 +1344,11 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Qiang Han (Irene)</t>
+          <t>JIE ZOU</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>55000</v>
+        <v>50000</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1373,11 +1373,11 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Qiang Han (Irene)</t>
+          <t>JIE ZOU</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>45000</v>
+        <v>60000</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1402,11 +1402,11 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Qiang Han (Irene)</t>
+          <t>JIE ZOU</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>40000</v>
+        <v>60000</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1431,11 +1431,11 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Qiang Han (Irene)</t>
+          <t>JIE ZOU</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>45000</v>
+        <v>50000</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -1460,11 +1460,11 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Qiang Han (Irene)</t>
+          <t>JIE ZOU</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>55000</v>
+        <v>60000</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -1489,11 +1489,11 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Qiang Han (Irene)</t>
+          <t>JIE ZOU</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>50000</v>
+        <v>55000</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -1518,7 +1518,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Jerry Ge</t>
+          <t>Victor Yang</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -1547,11 +1547,11 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Jerry Ge</t>
+          <t>Victor Yang</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>50000</v>
+        <v>55000</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -1576,11 +1576,11 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Jerry Ge</t>
+          <t>Victor Yang</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -1605,11 +1605,11 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Jerry Ge</t>
+          <t>Victor Yang</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -1634,11 +1634,11 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Jerry Ge</t>
+          <t>Victor Yang</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -1663,11 +1663,11 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Jerry Ge</t>
+          <t>Victor Yang</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>50000</v>
+        <v>55000</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -1692,11 +1692,11 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Jerry Ge</t>
+          <t>Victor Yang</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -1721,11 +1721,11 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Jerry Ge</t>
+          <t>Victor Yang</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -1750,11 +1750,11 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Jerry Ge</t>
+          <t>Victor Yang</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -1779,7 +1779,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Jerry Ge</t>
+          <t>Victor Yang</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Jerry Ge</t>
+          <t>Victor Yang</t>
         </is>
       </c>
       <c r="F48" t="n">
@@ -1837,7 +1837,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Jerry Ge</t>
+          <t>Victor Yang</t>
         </is>
       </c>
       <c r="F49" t="n">
@@ -1866,11 +1866,11 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Hao Yang (Emma)</t>
+          <t>Yan Wei (Emma)</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>115000</v>
+        <v>270000</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -1895,11 +1895,11 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Hao Yang (Emma)</t>
+          <t>Yan Wei (Emma)</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>115000</v>
+        <v>275000</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -1924,11 +1924,11 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Hao Yang (Emma)</t>
+          <t>Yan Wei (Emma)</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>125000</v>
+        <v>240000</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -1953,11 +1953,11 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Hao Yang (Emma)</t>
+          <t>Yan Wei (Emma)</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>120000</v>
+        <v>240000</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -1982,11 +1982,11 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Hao Yang (Emma)</t>
+          <t>Yan Wei (Emma)</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>135000</v>
+        <v>260000</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2011,11 +2011,11 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Hao Yang (Emma)</t>
+          <t>Yan Wei (Emma)</t>
         </is>
       </c>
       <c r="F55" t="n">
-        <v>120000</v>
+        <v>240000</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2040,11 +2040,11 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Hao Yang (Emma)</t>
+          <t>Yan Wei (Emma)</t>
         </is>
       </c>
       <c r="F56" t="n">
-        <v>110000</v>
+        <v>255000</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -2069,11 +2069,11 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Hao Yang (Emma)</t>
+          <t>Yan Wei (Emma)</t>
         </is>
       </c>
       <c r="F57" t="n">
-        <v>140000</v>
+        <v>260000</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -2098,11 +2098,11 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Hao Yang (Emma)</t>
+          <t>Yan Wei (Emma)</t>
         </is>
       </c>
       <c r="F58" t="n">
-        <v>110000</v>
+        <v>280000</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -2127,11 +2127,11 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Hao Yang (Emma)</t>
+          <t>Yan Wei (Emma)</t>
         </is>
       </c>
       <c r="F59" t="n">
-        <v>115000</v>
+        <v>270000</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -2156,11 +2156,11 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Hao Yang (Emma)</t>
+          <t>Yan Wei (Emma)</t>
         </is>
       </c>
       <c r="F60" t="n">
-        <v>110000</v>
+        <v>245000</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -2185,11 +2185,11 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Hao Yang (Emma)</t>
+          <t>Yan Wei (Emma)</t>
         </is>
       </c>
       <c r="F61" t="n">
-        <v>105000</v>
+        <v>220000</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -2214,7 +2214,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Mia Zou</t>
+          <t>Mia Xie</t>
         </is>
       </c>
       <c r="F62" t="n">
@@ -2243,11 +2243,11 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Mia Zou</t>
+          <t>Mia Xie</t>
         </is>
       </c>
       <c r="F63" t="n">
-        <v>80000</v>
+        <v>70000</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Mia Zou</t>
+          <t>Mia Xie</t>
         </is>
       </c>
       <c r="F64" t="n">
@@ -2301,11 +2301,11 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Mia Zou</t>
+          <t>Mia Xie</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>75000</v>
+        <v>85000</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -2330,11 +2330,11 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Mia Zou</t>
+          <t>Mia Xie</t>
         </is>
       </c>
       <c r="F66" t="n">
-        <v>85000</v>
+        <v>75000</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -2359,11 +2359,11 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Mia Zou</t>
+          <t>Mia Xie</t>
         </is>
       </c>
       <c r="F67" t="n">
-        <v>75000</v>
+        <v>85000</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -2388,11 +2388,11 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Mia Zou</t>
+          <t>Mia Xie</t>
         </is>
       </c>
       <c r="F68" t="n">
-        <v>70000</v>
+        <v>75000</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -2417,11 +2417,11 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Mia Zou</t>
+          <t>Mia Xie</t>
         </is>
       </c>
       <c r="F69" t="n">
-        <v>80000</v>
+        <v>75000</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -2446,7 +2446,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Mia Zou</t>
+          <t>Mia Xie</t>
         </is>
       </c>
       <c r="F70" t="n">
@@ -2475,11 +2475,11 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Mia Zou</t>
+          <t>Mia Xie</t>
         </is>
       </c>
       <c r="F71" t="n">
-        <v>75000</v>
+        <v>85000</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -2504,7 +2504,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Mia Zou</t>
+          <t>Mia Xie</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Mia Zou</t>
+          <t>Mia Xie</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -2562,11 +2562,11 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Lei Kong (Harvey)</t>
+          <t>Jason Zou</t>
         </is>
       </c>
       <c r="F74" t="n">
-        <v>35000</v>
+        <v>30000</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -2591,7 +2591,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Lei Kong (Harvey)</t>
+          <t>Jason Zou</t>
         </is>
       </c>
       <c r="F75" t="n">
@@ -2620,11 +2620,11 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Lei Kong (Harvey)</t>
+          <t>Jason Zou</t>
         </is>
       </c>
       <c r="F76" t="n">
-        <v>35000</v>
+        <v>30000</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -2649,11 +2649,11 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Lei Kong (Harvey)</t>
+          <t>Jason Zou</t>
         </is>
       </c>
       <c r="F77" t="n">
-        <v>40000</v>
+        <v>35000</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -2678,11 +2678,11 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Lei Kong (Harvey)</t>
+          <t>Jason Zou</t>
         </is>
       </c>
       <c r="F78" t="n">
-        <v>40000</v>
+        <v>35000</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -2707,11 +2707,11 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Lei Kong (Harvey)</t>
+          <t>Jason Zou</t>
         </is>
       </c>
       <c r="F79" t="n">
-        <v>30000</v>
+        <v>35000</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -2736,11 +2736,11 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Lei Kong (Harvey)</t>
+          <t>Jason Zou</t>
         </is>
       </c>
       <c r="F80" t="n">
-        <v>35000</v>
+        <v>30000</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -2765,7 +2765,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Lei Kong (Harvey)</t>
+          <t>Jason Zou</t>
         </is>
       </c>
       <c r="F81" t="n">
@@ -2794,11 +2794,11 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Lei Kong (Harvey)</t>
+          <t>Jason Zou</t>
         </is>
       </c>
       <c r="F82" t="n">
-        <v>35000</v>
+        <v>30000</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -2823,11 +2823,11 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Lei Kong (Harvey)</t>
+          <t>Jason Zou</t>
         </is>
       </c>
       <c r="F83" t="n">
-        <v>40000</v>
+        <v>30000</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -2852,11 +2852,11 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Lei Kong (Harvey)</t>
+          <t>Jason Zou</t>
         </is>
       </c>
       <c r="F84" t="n">
-        <v>35000</v>
+        <v>30000</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -2881,11 +2881,11 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Lei Kong (Harvey)</t>
+          <t>Jason Zou</t>
         </is>
       </c>
       <c r="F85" t="n">
-        <v>30000</v>
+        <v>35000</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -2910,11 +2910,11 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Ming Chu (Jerry)</t>
+          <t>YAN GE</t>
         </is>
       </c>
       <c r="F86" t="n">
-        <v>35000</v>
+        <v>70000</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -2939,11 +2939,11 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Ming Chu (Jerry)</t>
+          <t>YAN GE</t>
         </is>
       </c>
       <c r="F87" t="n">
-        <v>30000</v>
+        <v>80000</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -2968,11 +2968,11 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Ming Chu (Jerry)</t>
+          <t>YAN GE</t>
         </is>
       </c>
       <c r="F88" t="n">
-        <v>40000</v>
+        <v>65000</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -2997,11 +2997,11 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Ming Chu (Jerry)</t>
+          <t>YAN GE</t>
         </is>
       </c>
       <c r="F89" t="n">
-        <v>35000</v>
+        <v>70000</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -3026,11 +3026,11 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Ming Chu (Jerry)</t>
+          <t>YAN GE</t>
         </is>
       </c>
       <c r="F90" t="n">
-        <v>30000</v>
+        <v>75000</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -3055,11 +3055,11 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Ming Chu (Jerry)</t>
+          <t>YAN GE</t>
         </is>
       </c>
       <c r="F91" t="n">
-        <v>40000</v>
+        <v>70000</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -3084,11 +3084,11 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Ming Chu (Jerry)</t>
+          <t>YAN GE</t>
         </is>
       </c>
       <c r="F92" t="n">
-        <v>35000</v>
+        <v>80000</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -3113,11 +3113,11 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Ming Chu (Jerry)</t>
+          <t>YAN GE</t>
         </is>
       </c>
       <c r="F93" t="n">
-        <v>40000</v>
+        <v>65000</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -3142,11 +3142,11 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Ming Chu (Jerry)</t>
+          <t>YAN GE</t>
         </is>
       </c>
       <c r="F94" t="n">
-        <v>40000</v>
+        <v>65000</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -3171,11 +3171,11 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Ming Chu (Jerry)</t>
+          <t>YAN GE</t>
         </is>
       </c>
       <c r="F95" t="n">
-        <v>40000</v>
+        <v>75000</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -3200,11 +3200,11 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Ming Chu (Jerry)</t>
+          <t>YAN GE</t>
         </is>
       </c>
       <c r="F96" t="n">
-        <v>40000</v>
+        <v>80000</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -3229,11 +3229,11 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Ming Chu (Jerry)</t>
+          <t>YAN GE</t>
         </is>
       </c>
       <c r="F97" t="n">
-        <v>40000</v>
+        <v>75000</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -3258,11 +3258,11 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Rui Wei (Stella)</t>
+          <t>Amy Zou</t>
         </is>
       </c>
       <c r="F98" t="n">
-        <v>55000</v>
+        <v>65000</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -3287,11 +3287,11 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Rui Wei (Stella)</t>
+          <t>Amy Zou</t>
         </is>
       </c>
       <c r="F99" t="n">
-        <v>55000</v>
+        <v>75000</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -3316,11 +3316,11 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Rui Wei (Stella)</t>
+          <t>Amy Zou</t>
         </is>
       </c>
       <c r="F100" t="n">
-        <v>60000</v>
+        <v>70000</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -3345,11 +3345,11 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Rui Wei (Stella)</t>
+          <t>Amy Zou</t>
         </is>
       </c>
       <c r="F101" t="n">
-        <v>55000</v>
+        <v>80000</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -3374,11 +3374,11 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Rui Wei (Stella)</t>
+          <t>Amy Zou</t>
         </is>
       </c>
       <c r="F102" t="n">
-        <v>55000</v>
+        <v>60000</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -3403,11 +3403,11 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Rui Wei (Stella)</t>
+          <t>Amy Zou</t>
         </is>
       </c>
       <c r="F103" t="n">
-        <v>65000</v>
+        <v>60000</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -3432,11 +3432,11 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Rui Wei (Stella)</t>
+          <t>Amy Zou</t>
         </is>
       </c>
       <c r="F104" t="n">
-        <v>60000</v>
+        <v>75000</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
@@ -3461,7 +3461,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Rui Wei (Stella)</t>
+          <t>Amy Zou</t>
         </is>
       </c>
       <c r="F105" t="n">
@@ -3490,11 +3490,11 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Rui Wei (Stella)</t>
+          <t>Amy Zou</t>
         </is>
       </c>
       <c r="F106" t="n">
-        <v>70000</v>
+        <v>65000</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
@@ -3519,11 +3519,11 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Rui Wei (Stella)</t>
+          <t>Amy Zou</t>
         </is>
       </c>
       <c r="F107" t="n">
-        <v>60000</v>
+        <v>70000</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
@@ -3548,11 +3548,11 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Rui Wei (Stella)</t>
+          <t>Amy Zou</t>
         </is>
       </c>
       <c r="F108" t="n">
-        <v>70000</v>
+        <v>65000</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
@@ -3577,11 +3577,11 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Rui Wei (Stella)</t>
+          <t>Amy Zou</t>
         </is>
       </c>
       <c r="F109" t="n">
-        <v>70000</v>
+        <v>65000</v>
       </c>
       <c r="G109" t="inlineStr">
         <is>
@@ -3606,11 +3606,11 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>KAI ZHENG</t>
+          <t>Yun Zheng (Irene)</t>
         </is>
       </c>
       <c r="F110" t="n">
-        <v>30000</v>
+        <v>20000</v>
       </c>
       <c r="G110" t="inlineStr">
         <is>
@@ -3635,7 +3635,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>KAI ZHENG</t>
+          <t>Yun Zheng (Irene)</t>
         </is>
       </c>
       <c r="F111" t="n">
@@ -3664,11 +3664,11 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>KAI ZHENG</t>
+          <t>Yun Zheng (Irene)</t>
         </is>
       </c>
       <c r="F112" t="n">
-        <v>30000</v>
+        <v>25000</v>
       </c>
       <c r="G112" t="inlineStr">
         <is>
@@ -3693,11 +3693,11 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>KAI ZHENG</t>
+          <t>Yun Zheng (Irene)</t>
         </is>
       </c>
       <c r="F113" t="n">
-        <v>30000</v>
+        <v>25000</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
@@ -3722,7 +3722,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>KAI ZHENG</t>
+          <t>Yun Zheng (Irene)</t>
         </is>
       </c>
       <c r="F114" t="n">
@@ -3751,7 +3751,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>KAI ZHENG</t>
+          <t>Yun Zheng (Irene)</t>
         </is>
       </c>
       <c r="F115" t="n">
@@ -3780,7 +3780,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>KAI ZHENG</t>
+          <t>Yun Zheng (Irene)</t>
         </is>
       </c>
       <c r="F116" t="n">
@@ -3809,11 +3809,11 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>KAI ZHENG</t>
+          <t>Yun Zheng (Irene)</t>
         </is>
       </c>
       <c r="F117" t="n">
-        <v>30000</v>
+        <v>25000</v>
       </c>
       <c r="G117" t="inlineStr">
         <is>
@@ -3838,11 +3838,11 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>KAI ZHENG</t>
+          <t>Yun Zheng (Irene)</t>
         </is>
       </c>
       <c r="F118" t="n">
-        <v>30000</v>
+        <v>25000</v>
       </c>
       <c r="G118" t="inlineStr">
         <is>
@@ -3867,7 +3867,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>KAI ZHENG</t>
+          <t>Yun Zheng (Irene)</t>
         </is>
       </c>
       <c r="F119" t="n">
@@ -3896,11 +3896,11 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>KAI ZHENG</t>
+          <t>Yun Zheng (Irene)</t>
         </is>
       </c>
       <c r="F120" t="n">
-        <v>35000</v>
+        <v>25000</v>
       </c>
       <c r="G120" t="inlineStr">
         <is>
@@ -3925,7 +3925,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>KAI ZHENG</t>
+          <t>Yun Zheng (Irene)</t>
         </is>
       </c>
       <c r="F121" t="n">
@@ -3954,11 +3954,11 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Lei Ge (Tracy)</t>
+          <t>Peng He (Selina)</t>
         </is>
       </c>
       <c r="F122" t="n">
-        <v>25000</v>
+        <v>20000</v>
       </c>
       <c r="G122" t="inlineStr">
         <is>
@@ -3983,7 +3983,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Lei Ge (Tracy)</t>
+          <t>Peng He (Selina)</t>
         </is>
       </c>
       <c r="F123" t="n">
@@ -4012,11 +4012,11 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Lei Ge (Tracy)</t>
+          <t>Peng He (Selina)</t>
         </is>
       </c>
       <c r="F124" t="n">
-        <v>25000</v>
+        <v>20000</v>
       </c>
       <c r="G124" t="inlineStr">
         <is>
@@ -4041,11 +4041,11 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Lei Ge (Tracy)</t>
+          <t>Peng He (Selina)</t>
         </is>
       </c>
       <c r="F125" t="n">
-        <v>25000</v>
+        <v>20000</v>
       </c>
       <c r="G125" t="inlineStr">
         <is>
@@ -4070,7 +4070,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Lei Ge (Tracy)</t>
+          <t>Peng He (Selina)</t>
         </is>
       </c>
       <c r="F126" t="n">
@@ -4099,7 +4099,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Lei Ge (Tracy)</t>
+          <t>Peng He (Selina)</t>
         </is>
       </c>
       <c r="F127" t="n">
@@ -4128,11 +4128,11 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Lei Ge (Tracy)</t>
+          <t>Peng He (Selina)</t>
         </is>
       </c>
       <c r="F128" t="n">
-        <v>25000</v>
+        <v>20000</v>
       </c>
       <c r="G128" t="inlineStr">
         <is>
@@ -4157,7 +4157,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Lei Ge (Tracy)</t>
+          <t>Peng He (Selina)</t>
         </is>
       </c>
       <c r="F129" t="n">
@@ -4186,7 +4186,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Lei Ge (Tracy)</t>
+          <t>Peng He (Selina)</t>
         </is>
       </c>
       <c r="F130" t="n">
@@ -4215,7 +4215,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Lei Ge (Tracy)</t>
+          <t>Peng He (Selina)</t>
         </is>
       </c>
       <c r="F131" t="n">
@@ -4244,11 +4244,11 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Lei Ge (Tracy)</t>
+          <t>Peng He (Selina)</t>
         </is>
       </c>
       <c r="F132" t="n">
-        <v>25000</v>
+        <v>20000</v>
       </c>
       <c r="G132" t="inlineStr">
         <is>
@@ -4273,11 +4273,11 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Lei Ge (Tracy)</t>
+          <t>Peng He (Selina)</t>
         </is>
       </c>
       <c r="F133" t="n">
-        <v>25000</v>
+        <v>20000</v>
       </c>
       <c r="G133" t="inlineStr">
         <is>
@@ -4302,11 +4302,11 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>LAN WU</t>
+          <t>Hao Shi (Grace)</t>
         </is>
       </c>
       <c r="F134" t="n">
-        <v>115000</v>
+        <v>105000</v>
       </c>
       <c r="G134" t="inlineStr">
         <is>
@@ -4331,11 +4331,11 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>LAN WU</t>
+          <t>Hao Shi (Grace)</t>
         </is>
       </c>
       <c r="F135" t="n">
-        <v>115000</v>
+        <v>110000</v>
       </c>
       <c r="G135" t="inlineStr">
         <is>
@@ -4360,11 +4360,11 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>LAN WU</t>
+          <t>Hao Shi (Grace)</t>
         </is>
       </c>
       <c r="F136" t="n">
-        <v>110000</v>
+        <v>100000</v>
       </c>
       <c r="G136" t="inlineStr">
         <is>
@@ -4389,7 +4389,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>LAN WU</t>
+          <t>Hao Shi (Grace)</t>
         </is>
       </c>
       <c r="F137" t="n">
@@ -4418,11 +4418,11 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>LAN WU</t>
+          <t>Hao Shi (Grace)</t>
         </is>
       </c>
       <c r="F138" t="n">
-        <v>125000</v>
+        <v>95000</v>
       </c>
       <c r="G138" t="inlineStr">
         <is>
@@ -4447,11 +4447,11 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>LAN WU</t>
+          <t>Hao Shi (Grace)</t>
         </is>
       </c>
       <c r="F139" t="n">
-        <v>125000</v>
+        <v>110000</v>
       </c>
       <c r="G139" t="inlineStr">
         <is>
@@ -4476,11 +4476,11 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>LAN WU</t>
+          <t>Hao Shi (Grace)</t>
         </is>
       </c>
       <c r="F140" t="n">
-        <v>120000</v>
+        <v>110000</v>
       </c>
       <c r="G140" t="inlineStr">
         <is>
@@ -4505,7 +4505,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>LAN WU</t>
+          <t>Hao Shi (Grace)</t>
         </is>
       </c>
       <c r="F141" t="n">
@@ -4534,11 +4534,11 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>LAN WU</t>
+          <t>Hao Shi (Grace)</t>
         </is>
       </c>
       <c r="F142" t="n">
-        <v>105000</v>
+        <v>95000</v>
       </c>
       <c r="G142" t="inlineStr">
         <is>
@@ -4563,11 +4563,11 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>LAN WU</t>
+          <t>Hao Shi (Grace)</t>
         </is>
       </c>
       <c r="F143" t="n">
-        <v>115000</v>
+        <v>90000</v>
       </c>
       <c r="G143" t="inlineStr">
         <is>
@@ -4592,7 +4592,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>LAN WU</t>
+          <t>Hao Shi (Grace)</t>
         </is>
       </c>
       <c r="F144" t="n">
@@ -4621,11 +4621,11 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>LAN WU</t>
+          <t>Hao Shi (Grace)</t>
         </is>
       </c>
       <c r="F145" t="n">
-        <v>120000</v>
+        <v>110000</v>
       </c>
       <c r="G145" t="inlineStr">
         <is>
@@ -4655,88 +4655,88 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>8月任务</t>
+          <t>Aug Target</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>9月任务</t>
+          <t>Sep Target</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Lei He (Lina)</t>
+          <t>Cathy Kong</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>35000</v>
+        <v>25000</v>
       </c>
       <c r="C2" t="n">
-        <v>40000</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ting Qin (Joyce)</t>
+          <t>YUN CHU</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>90000</v>
+        <v>80000</v>
       </c>
       <c r="C3" t="n">
-        <v>105000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Qiang Han (Irene)</t>
+          <t>JIE ZOU</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>45000</v>
+        <v>60000</v>
       </c>
       <c r="C4" t="n">
-        <v>40000</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Jerry Ge</t>
+          <t>Victor Yang</t>
         </is>
       </c>
       <c r="B5" t="n">
+        <v>60000</v>
+      </c>
+      <c r="C5" t="n">
         <v>50000</v>
-      </c>
-      <c r="C5" t="n">
-        <v>60000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Hao Yang (Emma)</t>
+          <t>Yan Wei (Emma)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>140000</v>
+        <v>260000</v>
       </c>
       <c r="C6" t="n">
-        <v>110000</v>
+        <v>280000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Mia Zou</t>
+          <t>Mia Xie</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>80000</v>
+        <v>75000</v>
       </c>
       <c r="C7" t="n">
         <v>85000</v>
@@ -4745,59 +4745,59 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Lei Kong (Harvey)</t>
+          <t>Jason Zou</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>35000</v>
       </c>
       <c r="C8" t="n">
-        <v>35000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ming Chu (Jerry)</t>
+          <t>YAN GE</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>40000</v>
+        <v>65000</v>
       </c>
       <c r="C9" t="n">
-        <v>40000</v>
+        <v>65000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Rui Wei (Stella)</t>
+          <t>Amy Zou</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>70000</v>
       </c>
       <c r="C10" t="n">
-        <v>70000</v>
+        <v>65000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>KAI ZHENG</t>
+          <t>Yun Zheng (Irene)</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>30000</v>
+        <v>25000</v>
       </c>
       <c r="C11" t="n">
-        <v>30000</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Lei Ge (Tracy)</t>
+          <t>Peng He (Selina)</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -4810,14 +4810,14 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LAN WU</t>
+          <t>Hao Shi (Grace)</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>105000</v>
       </c>
       <c r="C13" t="n">
-        <v>105000</v>
+        <v>95000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>